<commit_message>
Latest Update for hosting
</commit_message>
<xml_diff>
--- a/Final_Menu_Categories_Products.xlsx
+++ b/Final_Menu_Categories_Products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\finalVDPFWebsite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EBEDFFF-B08C-4D7F-891B-5771718347A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A6FDDF-261E-4592-9B0B-3011570EDB61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,12 +17,15 @@
     <sheet name="Main &amp; Sub Categories" sheetId="2" r:id="rId2"/>
     <sheet name="All Products Mapping" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Products Mapping'!$A$1:$C$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="311">
   <si>
     <t>Main Category</t>
   </si>
@@ -193,9 +196,6 @@
   </si>
   <si>
     <t>Pongal</t>
-  </si>
-  <si>
-    <t>BB</t>
   </si>
   <si>
     <t>Palak Dal</t>
@@ -1322,6 +1322,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1721,11 +1724,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C264"/>
+  <dimension ref="A1:C263"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.453125" customWidth="1"/>
-    <col min="2" max="2" width="36.1796875" customWidth="1"/>
+    <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="83.6328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1968,7 +1971,7 @@
         <v>22</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>296</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -1979,7 +1982,7 @@
         <v>22</v>
       </c>
       <c r="C23" t="s">
-        <v>297</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -1998,7 +2001,7 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C25" t="s">
         <v>76</v>
@@ -2039,10 +2042,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C29" t="s">
         <v>80</v>
@@ -2163,7 +2166,7 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C40" t="s">
         <v>91</v>
@@ -2358,10 +2361,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C58" t="s">
         <v>109</v>
@@ -2427,7 +2430,7 @@
         <v>3</v>
       </c>
       <c r="B64" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C64" t="s">
         <v>115</v>
@@ -2743,21 +2746,21 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C93" t="s">
-        <v>144</v>
+        <v>28</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B94" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="C94" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
@@ -2963,7 +2966,7 @@
         <v>5</v>
       </c>
       <c r="B113" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C113" t="s">
         <v>163</v>
@@ -3029,7 +3032,7 @@
         <v>5</v>
       </c>
       <c r="B119" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C119" t="s">
         <v>169</v>
@@ -3103,10 +3106,10 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B126" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C126" t="s">
         <v>176</v>
@@ -3125,10 +3128,10 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B128" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C128" t="s">
         <v>178</v>
@@ -3235,10 +3238,10 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B138" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C138" t="s">
         <v>188</v>
@@ -3425,7 +3428,7 @@
         <v>8</v>
       </c>
       <c r="B155" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C155" t="s">
         <v>205</v>
@@ -3466,10 +3469,10 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B159" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C159" t="s">
         <v>209</v>
@@ -3532,10 +3535,10 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B165" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C165" t="s">
         <v>215</v>
@@ -3560,7 +3563,7 @@
         <v>10</v>
       </c>
       <c r="C167" t="s">
-        <v>217</v>
+        <v>305</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.35">
@@ -3571,7 +3574,7 @@
         <v>10</v>
       </c>
       <c r="C168" t="s">
-        <v>306</v>
+        <v>217</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.35">
@@ -3631,10 +3634,10 @@
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B174" t="s">
-        <v>10</v>
+        <v>310</v>
       </c>
       <c r="C174" t="s">
         <v>223</v>
@@ -3645,7 +3648,7 @@
         <v>11</v>
       </c>
       <c r="B175" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C175" t="s">
         <v>224</v>
@@ -3656,7 +3659,7 @@
         <v>11</v>
       </c>
       <c r="B176" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C176" t="s">
         <v>225</v>
@@ -3667,7 +3670,7 @@
         <v>11</v>
       </c>
       <c r="B177" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C177" t="s">
         <v>226</v>
@@ -3678,7 +3681,7 @@
         <v>11</v>
       </c>
       <c r="B178" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C178" t="s">
         <v>227</v>
@@ -3689,7 +3692,7 @@
         <v>11</v>
       </c>
       <c r="B179" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C179" t="s">
         <v>228</v>
@@ -3700,7 +3703,7 @@
         <v>11</v>
       </c>
       <c r="B180" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C180" t="s">
         <v>229</v>
@@ -3711,7 +3714,7 @@
         <v>11</v>
       </c>
       <c r="B181" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C181" t="s">
         <v>230</v>
@@ -3722,10 +3725,7 @@
         <v>11</v>
       </c>
       <c r="B182" t="s">
-        <v>311</v>
-      </c>
-      <c r="C182" t="s">
-        <v>231</v>
+        <v>38</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.35">
@@ -3733,7 +3733,10 @@
         <v>11</v>
       </c>
       <c r="B183" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="C183" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.35">
@@ -3771,13 +3774,10 @@
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B187" t="s">
-        <v>39</v>
-      </c>
-      <c r="C187" t="s">
-        <v>235</v>
+        <v>40</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.35">
@@ -3785,15 +3785,18 @@
         <v>12</v>
       </c>
       <c r="B188" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B189" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="C189" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.35">
@@ -3856,7 +3859,7 @@
         <v>13</v>
       </c>
       <c r="B195" t="s">
-        <v>42</v>
+        <v>304</v>
       </c>
       <c r="C195" t="s">
         <v>241</v>
@@ -3867,7 +3870,7 @@
         <v>13</v>
       </c>
       <c r="B196" t="s">
-        <v>305</v>
+        <v>42</v>
       </c>
       <c r="C196" t="s">
         <v>242</v>
@@ -3878,21 +3881,21 @@
         <v>13</v>
       </c>
       <c r="B197" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C197" t="s">
-        <v>243</v>
+        <v>43</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B198" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C198" t="s">
-        <v>43</v>
+        <v>306</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.35">
@@ -3919,13 +3922,13 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B201" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C201" t="s">
-        <v>309</v>
+        <v>243</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.35">
@@ -3963,10 +3966,10 @@
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B205" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C205" t="s">
         <v>247</v>
@@ -3991,7 +3994,7 @@
         <v>46</v>
       </c>
       <c r="C207" t="s">
-        <v>249</v>
+        <v>209</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.35">
@@ -4002,7 +4005,7 @@
         <v>46</v>
       </c>
       <c r="C208" t="s">
-        <v>210</v>
+        <v>249</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.35">
@@ -4128,10 +4131,10 @@
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B220" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C220" t="s">
         <v>261</v>
@@ -4230,7 +4233,7 @@
         <v>17</v>
       </c>
       <c r="B229" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C229" t="s">
         <v>270</v>
@@ -4271,10 +4274,10 @@
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B233" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C233" t="s">
         <v>274</v>
@@ -4392,10 +4395,10 @@
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B244" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C244" t="s">
         <v>285</v>
@@ -4519,7 +4522,7 @@
         <v>50</v>
       </c>
       <c r="C255" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.35">
@@ -4527,10 +4530,7 @@
         <v>19</v>
       </c>
       <c r="B256" t="s">
-        <v>50</v>
-      </c>
-      <c r="C256" t="s">
-        <v>298</v>
+        <v>51</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.35">
@@ -4538,7 +4538,10 @@
         <v>19</v>
       </c>
       <c r="B257" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="C257" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.35">
@@ -4554,10 +4557,10 @@
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B259" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C259" t="s">
         <v>300</v>
@@ -4571,7 +4574,7 @@
         <v>20</v>
       </c>
       <c r="C260" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.35">
@@ -4582,7 +4585,7 @@
         <v>20</v>
       </c>
       <c r="C261" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.35">
@@ -4607,18 +4610,8 @@
         <v>303</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A264" t="s">
-        <v>20</v>
-      </c>
-      <c r="B264" t="s">
-        <v>20</v>
-      </c>
-      <c r="C264" t="s">
-        <v>304</v>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>